<commit_message>
data(light-cones): G01-P7-L02 import light cone partition 02
</commit_message>
<xml_diff>
--- a/config/data/LightCone.xlsx
+++ b/config/data/LightCone.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -955,6 +955,342 @@
         <v>210016</v>
       </c>
     </row>
+    <row r="24">
+      <c r="B24" t="n">
+        <v>128</v>
+      </c>
+      <c r="C24" t="n">
+        <v>5</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Destruction</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>220001</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" t="n">
+        <v>129</v>
+      </c>
+      <c r="C25" t="n">
+        <v>5</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Harmony</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>220002</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" t="n">
+        <v>130</v>
+      </c>
+      <c r="C26" t="n">
+        <v>4</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Harmony</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>220003</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" t="n">
+        <v>131</v>
+      </c>
+      <c r="C27" t="n">
+        <v>3</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Harmony</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>220004</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" t="n">
+        <v>132</v>
+      </c>
+      <c r="C28" t="n">
+        <v>3</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Destruction</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>220005</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" t="n">
+        <v>133</v>
+      </c>
+      <c r="C29" t="n">
+        <v>4</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Preservation</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>220006</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" t="n">
+        <v>134</v>
+      </c>
+      <c r="C30" t="n">
+        <v>3</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Abundance</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>220007</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" t="n">
+        <v>135</v>
+      </c>
+      <c r="C31" t="n">
+        <v>5</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Hunt</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>220008</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" t="n">
+        <v>136</v>
+      </c>
+      <c r="C32" t="n">
+        <v>5</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Destruction</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>220009</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" t="n">
+        <v>137</v>
+      </c>
+      <c r="C33" t="n">
+        <v>4</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Harmony</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>220010</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" t="n">
+        <v>138</v>
+      </c>
+      <c r="C34" t="n">
+        <v>3</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Hunt</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>220011</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" t="n">
+        <v>139</v>
+      </c>
+      <c r="C35" t="n">
+        <v>3</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Erudition</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>220012</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" t="n">
+        <v>140</v>
+      </c>
+      <c r="C36" t="n">
+        <v>4</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Preservation</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>220013</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" t="n">
+        <v>141</v>
+      </c>
+      <c r="C37" t="n">
+        <v>5</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Elation</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>220014</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" t="n">
+        <v>142</v>
+      </c>
+      <c r="C38" t="n">
+        <v>3</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Preservation</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>220015</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" t="n">
+        <v>143</v>
+      </c>
+      <c r="C39" t="n">
+        <v>4</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Preservation</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>220016</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
data(light-cones): G01-P7-L03 import light cone partition 03
</commit_message>
<xml_diff>
--- a/config/data/LightCone.xlsx
+++ b/config/data/LightCone.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J39"/>
+  <dimension ref="A1:J55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1291,6 +1291,342 @@
         <v>220016</v>
       </c>
     </row>
+    <row r="40">
+      <c r="B40" t="n">
+        <v>144</v>
+      </c>
+      <c r="C40" t="n">
+        <v>4</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Abundance</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>230001</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" t="n">
+        <v>145</v>
+      </c>
+      <c r="C41" t="n">
+        <v>4</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Harmony</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>230002</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" t="n">
+        <v>146</v>
+      </c>
+      <c r="C42" t="n">
+        <v>5</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Harmony</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>230003</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" t="n">
+        <v>147</v>
+      </c>
+      <c r="C43" t="n">
+        <v>5</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Abundance</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>230004</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" t="n">
+        <v>148</v>
+      </c>
+      <c r="C44" t="n">
+        <v>5</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Elation</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>230005</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" t="n">
+        <v>149</v>
+      </c>
+      <c r="C45" t="n">
+        <v>5</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Harmony</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>230006</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" t="n">
+        <v>150</v>
+      </c>
+      <c r="C46" t="n">
+        <v>5</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Erudition</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>230007</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" t="n">
+        <v>151</v>
+      </c>
+      <c r="C47" t="n">
+        <v>4</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Nihility</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>230008</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" t="n">
+        <v>152</v>
+      </c>
+      <c r="C48" t="n">
+        <v>4</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Nihility</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v>230009</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" t="n">
+        <v>153</v>
+      </c>
+      <c r="C49" t="n">
+        <v>4</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Hunt</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>230010</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" t="n">
+        <v>154</v>
+      </c>
+      <c r="C50" t="n">
+        <v>3</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Abundance</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>230011</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" t="n">
+        <v>155</v>
+      </c>
+      <c r="C51" t="n">
+        <v>5</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Destruction</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F51" t="n">
+        <v>230012</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" t="n">
+        <v>156</v>
+      </c>
+      <c r="C52" t="n">
+        <v>4</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Destruction</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F52" t="n">
+        <v>230013</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" t="n">
+        <v>157</v>
+      </c>
+      <c r="C53" t="n">
+        <v>5</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Erudition</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F53" t="n">
+        <v>230014</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" t="n">
+        <v>158</v>
+      </c>
+      <c r="C54" t="n">
+        <v>5</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Harmony</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F54" t="n">
+        <v>230015</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" t="n">
+        <v>159</v>
+      </c>
+      <c r="C55" t="n">
+        <v>4</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Remembrance</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F55" t="n">
+        <v>230016</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
data(light-cones): G01-P7-L04 import light cone partition 04
</commit_message>
<xml_diff>
--- a/config/data/LightCone.xlsx
+++ b/config/data/LightCone.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J55"/>
+  <dimension ref="A1:J71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1627,6 +1627,342 @@
         <v>230016</v>
       </c>
     </row>
+    <row r="56">
+      <c r="B56" t="n">
+        <v>160</v>
+      </c>
+      <c r="C56" t="n">
+        <v>4</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Harmony</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F56" t="n">
+        <v>240001</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" t="n">
+        <v>161</v>
+      </c>
+      <c r="C57" t="n">
+        <v>4</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Remembrance</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F57" t="n">
+        <v>240002</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" t="n">
+        <v>162</v>
+      </c>
+      <c r="C58" t="n">
+        <v>4</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Erudition</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F58" t="n">
+        <v>240003</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" t="n">
+        <v>163</v>
+      </c>
+      <c r="C59" t="n">
+        <v>4</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Nihility</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F59" t="n">
+        <v>240004</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" t="n">
+        <v>164</v>
+      </c>
+      <c r="C60" t="n">
+        <v>4</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Abundance</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F60" t="n">
+        <v>240005</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" t="n">
+        <v>165</v>
+      </c>
+      <c r="C61" t="n">
+        <v>3</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Nihility</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F61" t="n">
+        <v>240006</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" t="n">
+        <v>166</v>
+      </c>
+      <c r="C62" t="n">
+        <v>4</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Nihility</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F62" t="n">
+        <v>240007</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" t="n">
+        <v>167</v>
+      </c>
+      <c r="C63" t="n">
+        <v>5</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Destruction</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F63" t="n">
+        <v>240008</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" t="n">
+        <v>168</v>
+      </c>
+      <c r="C64" t="n">
+        <v>5</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Destruction</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F64" t="n">
+        <v>240009</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" t="n">
+        <v>169</v>
+      </c>
+      <c r="C65" t="n">
+        <v>5</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Hunt</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F65" t="n">
+        <v>240010</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" t="n">
+        <v>170</v>
+      </c>
+      <c r="C66" t="n">
+        <v>5</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Harmony</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F66" t="n">
+        <v>240011</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" t="n">
+        <v>171</v>
+      </c>
+      <c r="C67" t="n">
+        <v>4</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Harmony</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F67" t="n">
+        <v>240012</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" t="n">
+        <v>172</v>
+      </c>
+      <c r="C68" t="n">
+        <v>5</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Nihility</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F68" t="n">
+        <v>240013</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" t="n">
+        <v>173</v>
+      </c>
+      <c r="C69" t="n">
+        <v>5</v>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Hunt</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F69" t="n">
+        <v>240014</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" t="n">
+        <v>174</v>
+      </c>
+      <c r="C70" t="n">
+        <v>5</v>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Nihility</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F70" t="n">
+        <v>240015</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" t="n">
+        <v>175</v>
+      </c>
+      <c r="C71" t="n">
+        <v>4</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Destruction</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F71" t="n">
+        <v>240016</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
data(light-cones): G01-P7-L05 import light cone partition 05
</commit_message>
<xml_diff>
--- a/config/data/LightCone.xlsx
+++ b/config/data/LightCone.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J71"/>
+  <dimension ref="A1:J87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1963,6 +1963,342 @@
         <v>240016</v>
       </c>
     </row>
+    <row r="72">
+      <c r="B72" t="n">
+        <v>176</v>
+      </c>
+      <c r="C72" t="n">
+        <v>5</v>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Preservation</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F72" t="n">
+        <v>250001</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="B73" t="n">
+        <v>177</v>
+      </c>
+      <c r="C73" t="n">
+        <v>5</v>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Erudition</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F73" t="n">
+        <v>250002</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="B74" t="n">
+        <v>178</v>
+      </c>
+      <c r="C74" t="n">
+        <v>4</v>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Nihility</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F74" t="n">
+        <v>250003</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="B75" t="n">
+        <v>179</v>
+      </c>
+      <c r="C75" t="n">
+        <v>4</v>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Preservation</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F75" t="n">
+        <v>250004</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="B76" t="n">
+        <v>180</v>
+      </c>
+      <c r="C76" t="n">
+        <v>4</v>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Preservation</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F76" t="n">
+        <v>250005</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="B77" t="n">
+        <v>181</v>
+      </c>
+      <c r="C77" t="n">
+        <v>5</v>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Nihility</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F77" t="n">
+        <v>250006</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="B78" t="n">
+        <v>182</v>
+      </c>
+      <c r="C78" t="n">
+        <v>5</v>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Erudition</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F78" t="n">
+        <v>250007</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="B79" t="n">
+        <v>183</v>
+      </c>
+      <c r="C79" t="n">
+        <v>3</v>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Elation</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F79" t="n">
+        <v>250008</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="B80" t="n">
+        <v>184</v>
+      </c>
+      <c r="C80" t="n">
+        <v>5</v>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Remembrance</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F80" t="n">
+        <v>250009</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="B81" t="n">
+        <v>185</v>
+      </c>
+      <c r="C81" t="n">
+        <v>5</v>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Nihility</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F81" t="n">
+        <v>250010</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="B82" t="n">
+        <v>186</v>
+      </c>
+      <c r="C82" t="n">
+        <v>3</v>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Nihility</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F82" t="n">
+        <v>250011</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="B83" t="n">
+        <v>187</v>
+      </c>
+      <c r="C83" t="n">
+        <v>5</v>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Remembrance</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F83" t="n">
+        <v>250012</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="B84" t="n">
+        <v>188</v>
+      </c>
+      <c r="C84" t="n">
+        <v>4</v>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Erudition</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F84" t="n">
+        <v>250013</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="B85" t="n">
+        <v>189</v>
+      </c>
+      <c r="C85" t="n">
+        <v>3</v>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Harmony</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F85" t="n">
+        <v>250014</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="B86" t="n">
+        <v>190</v>
+      </c>
+      <c r="C86" t="n">
+        <v>4</v>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Harmony</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F86" t="n">
+        <v>250015</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="B87" t="n">
+        <v>191</v>
+      </c>
+      <c r="C87" t="n">
+        <v>5</v>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Remembrance</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F87" t="n">
+        <v>250016</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
data(light-cones): G01-P7-L06 import light cone partition 06
</commit_message>
<xml_diff>
--- a/config/data/LightCone.xlsx
+++ b/config/data/LightCone.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J87"/>
+  <dimension ref="A1:J103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2299,6 +2299,342 @@
         <v>250016</v>
       </c>
     </row>
+    <row r="88">
+      <c r="B88" t="n">
+        <v>192</v>
+      </c>
+      <c r="C88" t="n">
+        <v>3</v>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Harmony</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F88" t="n">
+        <v>260001</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="B89" t="n">
+        <v>193</v>
+      </c>
+      <c r="C89" t="n">
+        <v>5</v>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Preservation</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F89" t="n">
+        <v>260002</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="B90" t="n">
+        <v>194</v>
+      </c>
+      <c r="C90" t="n">
+        <v>3</v>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Abundance</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F90" t="n">
+        <v>260003</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="B91" t="n">
+        <v>195</v>
+      </c>
+      <c r="C91" t="n">
+        <v>4</v>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Elation</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F91" t="n">
+        <v>260004</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="B92" t="n">
+        <v>196</v>
+      </c>
+      <c r="C92" t="n">
+        <v>3</v>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Destruction</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F92" t="n">
+        <v>260005</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="B93" t="n">
+        <v>197</v>
+      </c>
+      <c r="C93" t="n">
+        <v>5</v>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Nihility</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F93" t="n">
+        <v>260006</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="B94" t="n">
+        <v>198</v>
+      </c>
+      <c r="C94" t="n">
+        <v>5</v>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Abundance</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F94" t="n">
+        <v>260007</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="B95" t="n">
+        <v>199</v>
+      </c>
+      <c r="C95" t="n">
+        <v>5</v>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Erudition</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F95" t="n">
+        <v>260008</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="B96" t="n">
+        <v>200</v>
+      </c>
+      <c r="C96" t="n">
+        <v>4</v>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Destruction</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F96" t="n">
+        <v>260009</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="B97" t="n">
+        <v>201</v>
+      </c>
+      <c r="C97" t="n">
+        <v>5</v>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Erudition</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F97" t="n">
+        <v>260010</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="B98" t="n">
+        <v>202</v>
+      </c>
+      <c r="C98" t="n">
+        <v>4</v>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Destruction</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F98" t="n">
+        <v>260011</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="B99" t="n">
+        <v>203</v>
+      </c>
+      <c r="C99" t="n">
+        <v>5</v>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Destruction</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F99" t="n">
+        <v>260012</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="B100" t="n">
+        <v>204</v>
+      </c>
+      <c r="C100" t="n">
+        <v>4</v>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Hunt</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F100" t="n">
+        <v>260013</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="B101" t="n">
+        <v>205</v>
+      </c>
+      <c r="C101" t="n">
+        <v>3</v>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Erudition</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F101" t="n">
+        <v>260014</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="B102" t="n">
+        <v>206</v>
+      </c>
+      <c r="C102" t="n">
+        <v>4</v>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Harmony</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F102" t="n">
+        <v>260015</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="B103" t="n">
+        <v>207</v>
+      </c>
+      <c r="C103" t="n">
+        <v>5</v>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Harmony</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F103" t="n">
+        <v>260016</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
data(light-cones): G01-P7-L07 import light cone partition 07
</commit_message>
<xml_diff>
--- a/config/data/LightCone.xlsx
+++ b/config/data/LightCone.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J103"/>
+  <dimension ref="A1:J119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2635,6 +2635,342 @@
         <v>260016</v>
       </c>
     </row>
+    <row r="104">
+      <c r="B104" t="n">
+        <v>208</v>
+      </c>
+      <c r="C104" t="n">
+        <v>5</v>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Nihility</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F104" t="n">
+        <v>270001</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="B105" t="n">
+        <v>209</v>
+      </c>
+      <c r="C105" t="n">
+        <v>4</v>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Abundance</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F105" t="n">
+        <v>270002</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="B106" t="n">
+        <v>210</v>
+      </c>
+      <c r="C106" t="n">
+        <v>3</v>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Preservation</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F106" t="n">
+        <v>270003</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="B107" t="n">
+        <v>211</v>
+      </c>
+      <c r="C107" t="n">
+        <v>4</v>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Harmony</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F107" t="n">
+        <v>270004</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="B108" t="n">
+        <v>212</v>
+      </c>
+      <c r="C108" t="n">
+        <v>4</v>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Harmony</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F108" t="n">
+        <v>270005</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="B109" t="n">
+        <v>213</v>
+      </c>
+      <c r="C109" t="n">
+        <v>4</v>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Abundance</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F109" t="n">
+        <v>270006</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="B110" t="n">
+        <v>214</v>
+      </c>
+      <c r="C110" t="n">
+        <v>4</v>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Abundance</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F110" t="n">
+        <v>270007</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="B111" t="n">
+        <v>215</v>
+      </c>
+      <c r="C111" t="n">
+        <v>5</v>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Nihility</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F111" t="n">
+        <v>270008</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="B112" t="n">
+        <v>216</v>
+      </c>
+      <c r="C112" t="n">
+        <v>5</v>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Nihility</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F112" t="n">
+        <v>270009</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="B113" t="n">
+        <v>217</v>
+      </c>
+      <c r="C113" t="n">
+        <v>3</v>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Remembrance</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F113" t="n">
+        <v>270010</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="B114" t="n">
+        <v>218</v>
+      </c>
+      <c r="C114" t="n">
+        <v>4</v>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Nihility</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F114" t="n">
+        <v>270011</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="B115" t="n">
+        <v>219</v>
+      </c>
+      <c r="C115" t="n">
+        <v>4</v>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Hunt</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F115" t="n">
+        <v>270012</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="B116" t="n">
+        <v>220</v>
+      </c>
+      <c r="C116" t="n">
+        <v>4</v>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Hunt</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F116" t="n">
+        <v>270013</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="B117" t="n">
+        <v>221</v>
+      </c>
+      <c r="C117" t="n">
+        <v>3</v>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Erudition</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F117" t="n">
+        <v>270014</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="B118" t="n">
+        <v>222</v>
+      </c>
+      <c r="C118" t="n">
+        <v>5</v>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Hunt</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F118" t="n">
+        <v>270015</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="B119" t="n">
+        <v>223</v>
+      </c>
+      <c r="C119" t="n">
+        <v>5</v>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Abundance</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F119" t="n">
+        <v>270016</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
data(light-cones): G01-P7-L08 import light cone partition 08
</commit_message>
<xml_diff>
--- a/config/data/LightCone.xlsx
+++ b/config/data/LightCone.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J119"/>
+  <dimension ref="A1:J135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2971,6 +2971,342 @@
         <v>270016</v>
       </c>
     </row>
+    <row r="120">
+      <c r="B120" t="n">
+        <v>224</v>
+      </c>
+      <c r="C120" t="n">
+        <v>4</v>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Hunt</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F120" t="n">
+        <v>280001</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="B121" t="n">
+        <v>225</v>
+      </c>
+      <c r="C121" t="n">
+        <v>3</v>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Remembrance</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F121" t="n">
+        <v>280002</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="B122" t="n">
+        <v>226</v>
+      </c>
+      <c r="C122" t="n">
+        <v>4</v>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Hunt</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F122" t="n">
+        <v>280003</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="B123" t="n">
+        <v>227</v>
+      </c>
+      <c r="C123" t="n">
+        <v>4</v>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Abundance</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F123" t="n">
+        <v>280004</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="B124" t="n">
+        <v>228</v>
+      </c>
+      <c r="C124" t="n">
+        <v>3</v>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Destruction</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F124" t="n">
+        <v>280005</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="B125" t="n">
+        <v>229</v>
+      </c>
+      <c r="C125" t="n">
+        <v>5</v>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Preservation</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F125" t="n">
+        <v>280006</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="B126" t="n">
+        <v>230</v>
+      </c>
+      <c r="C126" t="n">
+        <v>5</v>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Hunt</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F126" t="n">
+        <v>280007</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="B127" t="n">
+        <v>231</v>
+      </c>
+      <c r="C127" t="n">
+        <v>3</v>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Elation</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F127" t="n">
+        <v>280008</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="B128" t="n">
+        <v>232</v>
+      </c>
+      <c r="C128" t="n">
+        <v>5</v>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Nihility</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F128" t="n">
+        <v>280009</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="B129" t="n">
+        <v>233</v>
+      </c>
+      <c r="C129" t="n">
+        <v>5</v>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Destruction</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F129" t="n">
+        <v>280010</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="B130" t="n">
+        <v>234</v>
+      </c>
+      <c r="C130" t="n">
+        <v>4</v>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Hunt</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F130" t="n">
+        <v>280011</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="B131" t="n">
+        <v>235</v>
+      </c>
+      <c r="C131" t="n">
+        <v>4</v>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Remembrance</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F131" t="n">
+        <v>280012</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="B132" t="n">
+        <v>236</v>
+      </c>
+      <c r="C132" t="n">
+        <v>4</v>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Hunt</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F132" t="n">
+        <v>280013</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="B133" t="n">
+        <v>237</v>
+      </c>
+      <c r="C133" t="n">
+        <v>5</v>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Preservation</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F133" t="n">
+        <v>280014</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="B134" t="n">
+        <v>238</v>
+      </c>
+      <c r="C134" t="n">
+        <v>4</v>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Erudition</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F134" t="n">
+        <v>280015</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="B135" t="n">
+        <v>239</v>
+      </c>
+      <c r="C135" t="n">
+        <v>4</v>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Erudition</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F135" t="n">
+        <v>280016</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
data(light-cones): G01-P7-L09 import light cone partition 09
</commit_message>
<xml_diff>
--- a/config/data/LightCone.xlsx
+++ b/config/data/LightCone.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J135"/>
+  <dimension ref="A1:J151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3307,6 +3307,342 @@
         <v>280016</v>
       </c>
     </row>
+    <row r="136">
+      <c r="B136" t="n">
+        <v>240</v>
+      </c>
+      <c r="C136" t="n">
+        <v>5</v>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Hunt</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F136" t="n">
+        <v>290001</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="B137" t="n">
+        <v>241</v>
+      </c>
+      <c r="C137" t="n">
+        <v>4</v>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Remembrance</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F137" t="n">
+        <v>290002</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="B138" t="n">
+        <v>242</v>
+      </c>
+      <c r="C138" t="n">
+        <v>4</v>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Harmony</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F138" t="n">
+        <v>290003</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="B139" t="n">
+        <v>243</v>
+      </c>
+      <c r="C139" t="n">
+        <v>4</v>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Erudition</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F139" t="n">
+        <v>290004</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="B140" t="n">
+        <v>244</v>
+      </c>
+      <c r="C140" t="n">
+        <v>5</v>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Hunt</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F140" t="n">
+        <v>290005</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="B141" t="n">
+        <v>245</v>
+      </c>
+      <c r="C141" t="n">
+        <v>4</v>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Destruction</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F141" t="n">
+        <v>290006</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="B142" t="n">
+        <v>246</v>
+      </c>
+      <c r="C142" t="n">
+        <v>4</v>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Erudition</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F142" t="n">
+        <v>290007</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="B143" t="n">
+        <v>247</v>
+      </c>
+      <c r="C143" t="n">
+        <v>4</v>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Remembrance</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F143" t="n">
+        <v>290008</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="B144" t="n">
+        <v>248</v>
+      </c>
+      <c r="C144" t="n">
+        <v>5</v>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Destruction</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F144" t="n">
+        <v>290009</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="B145" t="n">
+        <v>249</v>
+      </c>
+      <c r="C145" t="n">
+        <v>4</v>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Preservation</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F145" t="n">
+        <v>290010</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="B146" t="n">
+        <v>250</v>
+      </c>
+      <c r="C146" t="n">
+        <v>5</v>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Remembrance</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F146" t="n">
+        <v>290011</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="B147" t="n">
+        <v>251</v>
+      </c>
+      <c r="C147" t="n">
+        <v>5</v>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Nihility</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F147" t="n">
+        <v>290012</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="B148" t="n">
+        <v>252</v>
+      </c>
+      <c r="C148" t="n">
+        <v>5</v>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Preservation</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F148" t="n">
+        <v>290013</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="B149" t="n">
+        <v>253</v>
+      </c>
+      <c r="C149" t="n">
+        <v>5</v>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Destruction</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F149" t="n">
+        <v>290014</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="B150" t="n">
+        <v>254</v>
+      </c>
+      <c r="C150" t="n">
+        <v>5</v>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Abundance</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F150" t="n">
+        <v>290015</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="B151" t="n">
+        <v>255</v>
+      </c>
+      <c r="C151" t="n">
+        <v>5</v>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Remembrance</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F151" t="n">
+        <v>290016</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
data(light-cones): G01-P7-L10 import light cone partition 10
</commit_message>
<xml_diff>
--- a/config/data/LightCone.xlsx
+++ b/config/data/LightCone.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J151"/>
+  <dimension ref="A1:J167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3643,6 +3643,342 @@
         <v>290016</v>
       </c>
     </row>
+    <row r="152">
+      <c r="B152" t="n">
+        <v>256</v>
+      </c>
+      <c r="C152" t="n">
+        <v>5</v>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Remembrance</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F152" t="n">
+        <v>300001</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="B153" t="n">
+        <v>257</v>
+      </c>
+      <c r="C153" t="n">
+        <v>4</v>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Erudition</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F153" t="n">
+        <v>300002</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="B154" t="n">
+        <v>258</v>
+      </c>
+      <c r="C154" t="n">
+        <v>4</v>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Elation</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F154" t="n">
+        <v>300003</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="B155" t="n">
+        <v>259</v>
+      </c>
+      <c r="C155" t="n">
+        <v>4</v>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Elation</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F155" t="n">
+        <v>300004</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="B156" t="n">
+        <v>260</v>
+      </c>
+      <c r="C156" t="n">
+        <v>4</v>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Preservation</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F156" t="n">
+        <v>300005</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="B157" t="n">
+        <v>261</v>
+      </c>
+      <c r="C157" t="n">
+        <v>4</v>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Destruction</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F157" t="n">
+        <v>300006</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="B158" t="n">
+        <v>262</v>
+      </c>
+      <c r="C158" t="n">
+        <v>5</v>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Elation</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F158" t="n">
+        <v>300007</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="B159" t="n">
+        <v>263</v>
+      </c>
+      <c r="C159" t="n">
+        <v>4</v>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Abundance</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F159" t="n">
+        <v>300008</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="B160" t="n">
+        <v>264</v>
+      </c>
+      <c r="C160" t="n">
+        <v>4</v>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Remembrance</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F160" t="n">
+        <v>300009</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="B161" t="n">
+        <v>265</v>
+      </c>
+      <c r="C161" t="n">
+        <v>3</v>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Nihility</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F161" t="n">
+        <v>300010</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="B162" t="n">
+        <v>266</v>
+      </c>
+      <c r="C162" t="n">
+        <v>4</v>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Abundance</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F162" t="n">
+        <v>300011</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="B163" t="n">
+        <v>267</v>
+      </c>
+      <c r="C163" t="n">
+        <v>4</v>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Preservation</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F163" t="n">
+        <v>300012</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="B164" t="n">
+        <v>268</v>
+      </c>
+      <c r="C164" t="n">
+        <v>4</v>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Nihility</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F164" t="n">
+        <v>300013</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="B165" t="n">
+        <v>269</v>
+      </c>
+      <c r="C165" t="n">
+        <v>5</v>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Elation</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F165" t="n">
+        <v>300014</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="B166" t="n">
+        <v>270</v>
+      </c>
+      <c r="C166" t="n">
+        <v>4</v>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Abundance</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F166" t="n">
+        <v>300015</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="B167" t="n">
+        <v>271</v>
+      </c>
+      <c r="C167" t="n">
+        <v>5</v>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Elation</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F167" t="n">
+        <v>300016</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
data(light-cones): G01-P7-L11 import light cone partition 11
</commit_message>
<xml_diff>
--- a/config/data/LightCone.xlsx
+++ b/config/data/LightCone.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J167"/>
+  <dimension ref="A1:J172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3979,6 +3979,111 @@
         <v>300016</v>
       </c>
     </row>
+    <row r="168">
+      <c r="B168" t="n">
+        <v>272</v>
+      </c>
+      <c r="C168" t="n">
+        <v>5</v>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>Destruction</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F168" t="n">
+        <v>310001</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="B169" t="n">
+        <v>273</v>
+      </c>
+      <c r="C169" t="n">
+        <v>5</v>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Nihility</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F169" t="n">
+        <v>310002</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="B170" t="n">
+        <v>274</v>
+      </c>
+      <c r="C170" t="n">
+        <v>4</v>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Destruction</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F170" t="n">
+        <v>310003</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="B171" t="n">
+        <v>275</v>
+      </c>
+      <c r="C171" t="n">
+        <v>5</v>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Hunt</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F171" t="n">
+        <v>310004</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="B172" t="n">
+        <v>276</v>
+      </c>
+      <c r="C172" t="n">
+        <v>5</v>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Erudition</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>MatchingPath</t>
+        </is>
+      </c>
+      <c r="F172" t="n">
+        <v>310005</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>